<commit_message>
firwmare golve - upd 30/4
</commit_message>
<xml_diff>
--- a/Định nghĩa gói tin_tiến độ.xlsx
+++ b/Định nghĩa gói tin_tiến độ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Baitap\DATN\Smart_Glove\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5119A2E-C857-4D56-A0ED-87737E3765E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D13AF2B-AF90-47B6-81FD-4346C35F53B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D5384154-F6D8-428E-A6B5-0ECCAAE7B1F5}"/>
+    <workbookView xWindow="-28350" yWindow="2595" windowWidth="17280" windowHeight="11805" xr2:uid="{D5384154-F6D8-428E-A6B5-0ECCAAE7B1F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Trang_tính1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="59">
   <si>
     <t>cmd</t>
   </si>
@@ -111,9 +111,6 @@
     <t>"want": "tôi đau bụng"</t>
   </si>
   <si>
-    <t>Gửi lên BE đối với cử chỉ tay khẩn cấp</t>
-  </si>
-  <si>
     <t>"activity": 1,</t>
   </si>
   <si>
@@ -175,6 +172,48 @@
   </si>
   <si>
     <t>làm chương 1</t>
+  </si>
+  <si>
+    <t>Setup phone number</t>
+  </si>
+  <si>
+    <t>"phone_number":  "012345678"</t>
+  </si>
+  <si>
+    <t>Thay đổi số điện thoại gửi tin nhắn khẩn cấp</t>
+  </si>
+  <si>
+    <t>response connect to wifi successful</t>
+  </si>
+  <si>
+    <t>"ssid": "tên_wifi_của_bạn",</t>
+  </si>
+  <si>
+    <t>"ip": 192.168.1.2,</t>
+  </si>
+  <si>
+    <t>Địa chỉ io của esp32 được cấp sau khi kết nối wifi</t>
+  </si>
+  <si>
+    <t>connect_wifi</t>
+  </si>
+  <si>
+    <t>User gửi khi muốn ESP32  kết nối wifi</t>
+  </si>
+  <si>
+    <t>"ssid": "tên_wifi_của bạn"  ,</t>
+  </si>
+  <si>
+    <t>"password": "pass"</t>
+  </si>
+  <si>
+    <t>disconnect wifi</t>
+  </si>
+  <si>
+    <t>User gửi khi muốn ngắt kết nối wifi</t>
+  </si>
+  <si>
+    <t>Gửi lên backend mỗi khi nhận diện được cử chỉ tay tương ứng</t>
   </si>
 </sst>
 </file>
@@ -231,13 +270,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -574,7 +616,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{750ECDB7-2438-43E7-9C6F-4FD5B31CB47B}">
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.21875" bestFit="1" customWidth="1"/>
@@ -648,12 +690,12 @@
         <v>3</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C9" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
@@ -725,7 +767,7 @@
         <v>3</v>
       </c>
       <c r="D19" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -735,6 +777,117 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C21" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23">
+        <v>103</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C24" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C25" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27">
+        <v>203</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C28" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C29" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D29" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C30" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C31" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33">
+        <v>104</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D33" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C34" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C35" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C36" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>56</v>
+      </c>
+      <c r="B38">
+        <v>105</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D38" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C39" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C40" s="1" t="s">
         <v>6</v>
       </c>
     </row>
@@ -756,70 +909,70 @@
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>40</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>41</v>
       </c>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
smart glove - ready for testing
</commit_message>
<xml_diff>
--- a/Định nghĩa gói tin_tiến độ.xlsx
+++ b/Định nghĩa gói tin_tiến độ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Baitap\DATN\Smart_Glove\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{692D7655-57BC-4EDF-BC00-6D6F8D09B146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5364E252-B2A3-45E5-BEA8-7657721E622A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D5384154-F6D8-428E-A6B5-0ECCAAE7B1F5}"/>
   </bookViews>
@@ -69,12 +69,6 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>sub: SmartGlove/sub</t>
-  </si>
-  <si>
-    <t>pub: SmartGlove/pub</t>
-  </si>
-  <si>
     <t>1xx:sub</t>
   </si>
   <si>
@@ -214,13 +208,19 @@
   </si>
   <si>
     <t>Gửi lên backend mỗi khi nhận diện được cử chỉ tay tương ứng</t>
+  </si>
+  <si>
+    <t>sub: ESP32/sub</t>
+  </si>
+  <si>
+    <t>pub: ESP32/pub</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -234,16 +234,33 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -266,11 +283,79 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -279,9 +364,93 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
@@ -627,7 +796,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C1" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -639,18 +808,18 @@
         <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C2" t="s">
-        <v>11</v>
+        <v>58</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="K2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
@@ -669,229 +838,346 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="10">
+        <v>101</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="5"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="5"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="5"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="5"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="6"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="6"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="19">
+        <v>102</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="21"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="B8">
-        <v>101</v>
-      </c>
-      <c r="C8" s="1" t="s">
+      <c r="D13" s="21"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="24"/>
+      <c r="B14" s="25"/>
+      <c r="C14" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="24"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="27">
+        <v>201</v>
+      </c>
+      <c r="C15" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="D8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C9" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C10" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C11" s="1" t="s">
+      <c r="D15" s="26" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="29"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="31" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="29"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="29"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="31" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12">
-        <v>102</v>
-      </c>
-      <c r="C12" s="1" t="s">
+      <c r="D17" s="29"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="32"/>
+      <c r="B18" s="33"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="32"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="10">
+        <v>202</v>
+      </c>
+      <c r="C19" s="15" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C13" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="D19" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="5"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D20" s="5"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="5"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21" s="5"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="6"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="6"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" s="10">
+        <v>103</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="5"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" s="5"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="5"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="5"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="6"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="6"/>
+    </row>
+    <row r="27" spans="1:4" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" s="10">
+        <v>203</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="8"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="D28" s="5"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="8"/>
+      <c r="B29" s="11"/>
+      <c r="C29" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D29" s="5"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="8"/>
+      <c r="B30" s="11"/>
+      <c r="C30" s="16" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C14" s="1" t="s">
+      <c r="D30" s="5"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="8"/>
+      <c r="B31" s="11"/>
+      <c r="C31" s="16" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15">
-        <v>201</v>
-      </c>
-      <c r="C15" s="1" t="s">
+      <c r="D31" s="5"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="9"/>
+      <c r="B32" s="12"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="6"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B33" s="10">
+        <v>104</v>
+      </c>
+      <c r="C33" s="15" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C16" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C17" s="1" t="s">
+      <c r="D33" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="5"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="D34" s="5"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="5"/>
+      <c r="B35" s="11"/>
+      <c r="C35" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="D35" s="5"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="5"/>
+      <c r="B36" s="11"/>
+      <c r="C36" s="16" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>22</v>
-      </c>
-      <c r="B19">
-        <v>202</v>
-      </c>
-      <c r="C19" s="1" t="s">
+      <c r="D36" s="5"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="6"/>
+      <c r="B37" s="12"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="6"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B38" s="10">
+        <v>105</v>
+      </c>
+      <c r="C38" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="D19" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C20" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C21" s="1" t="s">
+      <c r="D38" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="5"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" s="5"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" s="6"/>
+      <c r="B40" s="12"/>
+      <c r="C40" s="14" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>45</v>
-      </c>
-      <c r="B23">
-        <v>103</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C24" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D24" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C25" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B27">
-        <v>203</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C28" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C29" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D29" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C30" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C31" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>52</v>
-      </c>
-      <c r="B33">
-        <v>104</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D33" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C34" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C35" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C36" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>56</v>
-      </c>
-      <c r="B38">
-        <v>105</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D38" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C39" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C40" s="1" t="s">
-        <v>6</v>
-      </c>
+      <c r="D40" s="6"/>
     </row>
   </sheetData>
+  <mergeCells count="24">
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="D8:D11"/>
+    <mergeCell ref="D12:D14"/>
+    <mergeCell ref="D15:D18"/>
+    <mergeCell ref="D19:D22"/>
+    <mergeCell ref="D23:D26"/>
+    <mergeCell ref="D27:D32"/>
+    <mergeCell ref="D33:D37"/>
+    <mergeCell ref="D38:D40"/>
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="B19:B22"/>
+    <mergeCell ref="A23:A26"/>
+    <mergeCell ref="A27:A32"/>
+    <mergeCell ref="A33:A37"/>
+    <mergeCell ref="A38:A40"/>
+    <mergeCell ref="B23:B26"/>
+    <mergeCell ref="B27:B32"/>
+    <mergeCell ref="B33:B37"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="B12:B14"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="B15:B18"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -909,70 +1195,70 @@
   <sheetData>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>38</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>40</v>
       </c>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>